<commit_message>
Frontend básico feito, chat respondendo com respostas genéricas. Interface feita com React e TypeScript.
</commit_message>
<xml_diff>
--- a/Projeto 1/dados.xlsx
+++ b/Projeto 1/dados.xlsx
@@ -2031,12 +2031,18 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -2066,11 +2072,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2375,6 +2385,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AA148"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="3.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="6.6640625" style="3" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -2449,13 +2487,13 @@
       <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2532,13 +2570,13 @@
       <c r="X2" t="s">
         <v>45</v>
       </c>
-      <c r="Y2">
-        <v>1</v>
-      </c>
-      <c r="Z2">
-        <v>1</v>
-      </c>
-      <c r="AA2">
+      <c r="Y2" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA2" s="3">
         <v>1</v>
       </c>
     </row>
@@ -2615,13 +2653,13 @@
       <c r="X3" t="s">
         <v>61</v>
       </c>
-      <c r="Y3">
-        <v>0</v>
-      </c>
-      <c r="Z3">
-        <v>0</v>
-      </c>
-      <c r="AA3">
+      <c r="Y3" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="3">
         <v>0</v>
       </c>
     </row>
@@ -2698,13 +2736,13 @@
       <c r="X4" t="s">
         <v>77</v>
       </c>
-      <c r="Y4">
-        <v>0</v>
-      </c>
-      <c r="Z4">
-        <v>0</v>
-      </c>
-      <c r="AA4">
+      <c r="Y4" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="3">
         <v>0</v>
       </c>
     </row>
@@ -2781,13 +2819,13 @@
       <c r="X5" t="s">
         <v>84</v>
       </c>
-      <c r="Y5">
-        <v>1</v>
-      </c>
-      <c r="Z5">
-        <v>1</v>
-      </c>
-      <c r="AA5">
+      <c r="Y5" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z5" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA5" s="3">
         <v>1</v>
       </c>
     </row>
@@ -2864,13 +2902,13 @@
       <c r="X6" t="s">
         <v>90</v>
       </c>
-      <c r="Y6">
-        <v>0</v>
-      </c>
-      <c r="Z6">
-        <v>0</v>
-      </c>
-      <c r="AA6">
+      <c r="Y6" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="3">
         <v>0</v>
       </c>
     </row>
@@ -2947,13 +2985,13 @@
       <c r="X7" t="s">
         <v>96</v>
       </c>
-      <c r="Y7">
-        <v>0</v>
-      </c>
-      <c r="Z7">
-        <v>0</v>
-      </c>
-      <c r="AA7">
+      <c r="Y7" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3030,13 +3068,13 @@
       <c r="X8" t="s">
         <v>102</v>
       </c>
-      <c r="Y8">
-        <v>1</v>
-      </c>
-      <c r="Z8">
-        <v>1</v>
-      </c>
-      <c r="AA8">
+      <c r="Y8" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA8" s="3">
         <v>1</v>
       </c>
     </row>
@@ -3113,13 +3151,13 @@
       <c r="X9" t="s">
         <v>107</v>
       </c>
-      <c r="Y9">
-        <v>0</v>
-      </c>
-      <c r="Z9">
-        <v>0</v>
-      </c>
-      <c r="AA9">
+      <c r="Y9" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA9" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3196,13 +3234,13 @@
       <c r="X10" t="s">
         <v>112</v>
       </c>
-      <c r="Y10">
-        <v>0</v>
-      </c>
-      <c r="Z10">
-        <v>0</v>
-      </c>
-      <c r="AA10">
+      <c r="Y10" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3279,13 +3317,13 @@
       <c r="X11" t="s">
         <v>116</v>
       </c>
-      <c r="Y11">
-        <v>1</v>
-      </c>
-      <c r="Z11">
-        <v>1</v>
-      </c>
-      <c r="AA11">
+      <c r="Y11" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z11" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA11" s="3">
         <v>1</v>
       </c>
     </row>
@@ -3362,13 +3400,13 @@
       <c r="X12" t="s">
         <v>120</v>
       </c>
-      <c r="Y12">
-        <v>0</v>
-      </c>
-      <c r="Z12">
-        <v>0</v>
-      </c>
-      <c r="AA12">
+      <c r="Y12" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3445,13 +3483,13 @@
       <c r="X13" t="s">
         <v>124</v>
       </c>
-      <c r="Y13">
-        <v>0</v>
-      </c>
-      <c r="Z13">
-        <v>0</v>
-      </c>
-      <c r="AA13">
+      <c r="Y13" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3528,13 +3566,13 @@
       <c r="X14" t="s">
         <v>128</v>
       </c>
-      <c r="Y14">
-        <v>1</v>
-      </c>
-      <c r="Z14">
-        <v>1</v>
-      </c>
-      <c r="AA14">
+      <c r="Y14" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z14" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA14" s="3">
         <v>1</v>
       </c>
     </row>
@@ -3611,13 +3649,13 @@
       <c r="X15" t="s">
         <v>132</v>
       </c>
-      <c r="Y15">
-        <v>0</v>
-      </c>
-      <c r="Z15">
-        <v>0</v>
-      </c>
-      <c r="AA15">
+      <c r="Y15" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3694,13 +3732,13 @@
       <c r="X16" t="s">
         <v>136</v>
       </c>
-      <c r="Y16">
-        <v>0</v>
-      </c>
-      <c r="Z16">
-        <v>0</v>
-      </c>
-      <c r="AA16">
+      <c r="Y16" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3777,13 +3815,13 @@
       <c r="X17" t="s">
         <v>140</v>
       </c>
-      <c r="Y17">
-        <v>1</v>
-      </c>
-      <c r="Z17">
-        <v>1</v>
-      </c>
-      <c r="AA17">
+      <c r="Y17" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z17" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA17" s="3">
         <v>1</v>
       </c>
     </row>
@@ -3860,13 +3898,13 @@
       <c r="X18" t="s">
         <v>144</v>
       </c>
-      <c r="Y18">
-        <v>0</v>
-      </c>
-      <c r="Z18">
-        <v>0</v>
-      </c>
-      <c r="AA18">
+      <c r="Y18" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z18" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA18" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3943,13 +3981,13 @@
       <c r="X19" t="s">
         <v>148</v>
       </c>
-      <c r="Y19">
-        <v>0</v>
-      </c>
-      <c r="Z19">
-        <v>0</v>
-      </c>
-      <c r="AA19">
+      <c r="Y19" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4026,13 +4064,13 @@
       <c r="X20" t="s">
         <v>152</v>
       </c>
-      <c r="Y20">
-        <v>1</v>
-      </c>
-      <c r="Z20">
-        <v>1</v>
-      </c>
-      <c r="AA20">
+      <c r="Y20" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z20" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA20" s="3">
         <v>1</v>
       </c>
     </row>
@@ -4109,13 +4147,13 @@
       <c r="X21" t="s">
         <v>156</v>
       </c>
-      <c r="Y21">
-        <v>0</v>
-      </c>
-      <c r="Z21">
-        <v>0</v>
-      </c>
-      <c r="AA21">
+      <c r="Y21" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA21" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4192,13 +4230,13 @@
       <c r="X22" t="s">
         <v>160</v>
       </c>
-      <c r="Y22">
-        <v>0</v>
-      </c>
-      <c r="Z22">
-        <v>0</v>
-      </c>
-      <c r="AA22">
+      <c r="Y22" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA22" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4275,13 +4313,13 @@
       <c r="X23" t="s">
         <v>164</v>
       </c>
-      <c r="Y23">
-        <v>1</v>
-      </c>
-      <c r="Z23">
-        <v>1</v>
-      </c>
-      <c r="AA23">
+      <c r="Y23" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z23" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA23" s="3">
         <v>1</v>
       </c>
     </row>
@@ -4358,13 +4396,13 @@
       <c r="X24" t="s">
         <v>168</v>
       </c>
-      <c r="Y24">
-        <v>0</v>
-      </c>
-      <c r="Z24">
-        <v>0</v>
-      </c>
-      <c r="AA24">
+      <c r="Y24" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z24" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA24" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4441,13 +4479,13 @@
       <c r="X25" t="s">
         <v>172</v>
       </c>
-      <c r="Y25">
-        <v>0</v>
-      </c>
-      <c r="Z25">
-        <v>0</v>
-      </c>
-      <c r="AA25">
+      <c r="Y25" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z25" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA25" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4524,13 +4562,13 @@
       <c r="X26" t="s">
         <v>176</v>
       </c>
-      <c r="Y26">
-        <v>1</v>
-      </c>
-      <c r="Z26">
-        <v>1</v>
-      </c>
-      <c r="AA26">
+      <c r="Y26" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z26" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA26" s="3">
         <v>1</v>
       </c>
     </row>
@@ -4607,13 +4645,13 @@
       <c r="X27" t="s">
         <v>180</v>
       </c>
-      <c r="Y27">
-        <v>0</v>
-      </c>
-      <c r="Z27">
-        <v>0</v>
-      </c>
-      <c r="AA27">
+      <c r="Y27" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z27" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA27" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4690,13 +4728,13 @@
       <c r="X28" t="s">
         <v>184</v>
       </c>
-      <c r="Y28">
-        <v>0</v>
-      </c>
-      <c r="Z28">
-        <v>0</v>
-      </c>
-      <c r="AA28">
+      <c r="Y28" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z28" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA28" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4773,13 +4811,13 @@
       <c r="X29" t="s">
         <v>188</v>
       </c>
-      <c r="Y29">
-        <v>1</v>
-      </c>
-      <c r="Z29">
-        <v>1</v>
-      </c>
-      <c r="AA29">
+      <c r="Y29" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z29" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA29" s="3">
         <v>1</v>
       </c>
     </row>
@@ -4856,13 +4894,13 @@
       <c r="X30" t="s">
         <v>192</v>
       </c>
-      <c r="Y30">
-        <v>0</v>
-      </c>
-      <c r="Z30">
-        <v>0</v>
-      </c>
-      <c r="AA30">
+      <c r="Y30" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA30" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4939,13 +4977,13 @@
       <c r="X31" t="s">
         <v>196</v>
       </c>
-      <c r="Y31">
-        <v>0</v>
-      </c>
-      <c r="Z31">
-        <v>0</v>
-      </c>
-      <c r="AA31">
+      <c r="Y31" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA31" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5022,13 +5060,13 @@
       <c r="X32" t="s">
         <v>200</v>
       </c>
-      <c r="Y32">
-        <v>1</v>
-      </c>
-      <c r="Z32">
-        <v>1</v>
-      </c>
-      <c r="AA32">
+      <c r="Y32" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z32" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA32" s="3">
         <v>1</v>
       </c>
     </row>
@@ -5105,13 +5143,13 @@
       <c r="X33" t="s">
         <v>204</v>
       </c>
-      <c r="Y33">
-        <v>0</v>
-      </c>
-      <c r="Z33">
-        <v>0</v>
-      </c>
-      <c r="AA33">
+      <c r="Y33" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA33" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5188,13 +5226,13 @@
       <c r="X34" t="s">
         <v>208</v>
       </c>
-      <c r="Y34">
-        <v>0</v>
-      </c>
-      <c r="Z34">
-        <v>0</v>
-      </c>
-      <c r="AA34">
+      <c r="Y34" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z34" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA34" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5271,13 +5309,13 @@
       <c r="X35" t="s">
         <v>212</v>
       </c>
-      <c r="Y35">
-        <v>1</v>
-      </c>
-      <c r="Z35">
-        <v>1</v>
-      </c>
-      <c r="AA35">
+      <c r="Y35" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z35" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA35" s="3">
         <v>1</v>
       </c>
     </row>
@@ -5354,13 +5392,13 @@
       <c r="X36" t="s">
         <v>216</v>
       </c>
-      <c r="Y36">
-        <v>0</v>
-      </c>
-      <c r="Z36">
-        <v>0</v>
-      </c>
-      <c r="AA36">
+      <c r="Y36" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z36" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA36" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5437,13 +5475,13 @@
       <c r="X37" t="s">
         <v>220</v>
       </c>
-      <c r="Y37">
-        <v>0</v>
-      </c>
-      <c r="Z37">
-        <v>0</v>
-      </c>
-      <c r="AA37">
+      <c r="Y37" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA37" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5520,13 +5558,13 @@
       <c r="X38" t="s">
         <v>224</v>
       </c>
-      <c r="Y38">
-        <v>1</v>
-      </c>
-      <c r="Z38">
-        <v>1</v>
-      </c>
-      <c r="AA38">
+      <c r="Y38" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z38" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA38" s="3">
         <v>1</v>
       </c>
     </row>
@@ -5603,13 +5641,13 @@
       <c r="X39" t="s">
         <v>228</v>
       </c>
-      <c r="Y39">
-        <v>0</v>
-      </c>
-      <c r="Z39">
-        <v>0</v>
-      </c>
-      <c r="AA39">
+      <c r="Y39" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA39" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5686,13 +5724,13 @@
       <c r="X40" t="s">
         <v>232</v>
       </c>
-      <c r="Y40">
-        <v>0</v>
-      </c>
-      <c r="Z40">
-        <v>0</v>
-      </c>
-      <c r="AA40">
+      <c r="Y40" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z40" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA40" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5769,13 +5807,13 @@
       <c r="X41" t="s">
         <v>236</v>
       </c>
-      <c r="Y41">
-        <v>1</v>
-      </c>
-      <c r="Z41">
-        <v>1</v>
-      </c>
-      <c r="AA41">
+      <c r="Y41" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z41" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA41" s="3">
         <v>1</v>
       </c>
     </row>
@@ -5852,13 +5890,13 @@
       <c r="X42" t="s">
         <v>240</v>
       </c>
-      <c r="Y42">
-        <v>0</v>
-      </c>
-      <c r="Z42">
-        <v>0</v>
-      </c>
-      <c r="AA42">
+      <c r="Y42" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z42" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA42" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5935,13 +5973,13 @@
       <c r="X43" t="s">
         <v>244</v>
       </c>
-      <c r="Y43">
-        <v>0</v>
-      </c>
-      <c r="Z43">
-        <v>0</v>
-      </c>
-      <c r="AA43">
+      <c r="Y43" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z43" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA43" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6018,13 +6056,13 @@
       <c r="X44" t="s">
         <v>248</v>
       </c>
-      <c r="Y44">
-        <v>1</v>
-      </c>
-      <c r="Z44">
-        <v>1</v>
-      </c>
-      <c r="AA44">
+      <c r="Y44" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z44" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA44" s="3">
         <v>1</v>
       </c>
     </row>
@@ -6101,13 +6139,13 @@
       <c r="X45" t="s">
         <v>252</v>
       </c>
-      <c r="Y45">
-        <v>0</v>
-      </c>
-      <c r="Z45">
-        <v>0</v>
-      </c>
-      <c r="AA45">
+      <c r="Y45" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z45" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA45" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6184,13 +6222,13 @@
       <c r="X46" t="s">
         <v>256</v>
       </c>
-      <c r="Y46">
-        <v>0</v>
-      </c>
-      <c r="Z46">
-        <v>0</v>
-      </c>
-      <c r="AA46">
+      <c r="Y46" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z46" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA46" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6267,13 +6305,13 @@
       <c r="X47" t="s">
         <v>260</v>
       </c>
-      <c r="Y47">
-        <v>1</v>
-      </c>
-      <c r="Z47">
-        <v>1</v>
-      </c>
-      <c r="AA47">
+      <c r="Y47" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z47" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA47" s="3">
         <v>1</v>
       </c>
     </row>
@@ -6350,13 +6388,13 @@
       <c r="X48" t="s">
         <v>264</v>
       </c>
-      <c r="Y48">
-        <v>0</v>
-      </c>
-      <c r="Z48">
-        <v>0</v>
-      </c>
-      <c r="AA48">
+      <c r="Y48" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z48" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA48" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6433,13 +6471,13 @@
       <c r="X49" t="s">
         <v>268</v>
       </c>
-      <c r="Y49">
-        <v>0</v>
-      </c>
-      <c r="Z49">
-        <v>0</v>
-      </c>
-      <c r="AA49">
+      <c r="Y49" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z49" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA49" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6516,13 +6554,13 @@
       <c r="X50" t="s">
         <v>272</v>
       </c>
-      <c r="Y50">
-        <v>1</v>
-      </c>
-      <c r="Z50">
-        <v>1</v>
-      </c>
-      <c r="AA50">
+      <c r="Y50" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z50" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA50" s="3">
         <v>1</v>
       </c>
     </row>
@@ -6599,13 +6637,13 @@
       <c r="X51" t="s">
         <v>276</v>
       </c>
-      <c r="Y51">
-        <v>0</v>
-      </c>
-      <c r="Z51">
-        <v>0</v>
-      </c>
-      <c r="AA51">
+      <c r="Y51" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z51" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA51" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6682,13 +6720,13 @@
       <c r="X52" t="s">
         <v>280</v>
       </c>
-      <c r="Y52">
-        <v>0</v>
-      </c>
-      <c r="Z52">
-        <v>0</v>
-      </c>
-      <c r="AA52">
+      <c r="Y52" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z52" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA52" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6765,13 +6803,13 @@
       <c r="X53" t="s">
         <v>284</v>
       </c>
-      <c r="Y53">
-        <v>1</v>
-      </c>
-      <c r="Z53">
-        <v>1</v>
-      </c>
-      <c r="AA53">
+      <c r="Y53" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z53" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA53" s="3">
         <v>1</v>
       </c>
     </row>
@@ -6848,13 +6886,13 @@
       <c r="X54" t="s">
         <v>288</v>
       </c>
-      <c r="Y54">
-        <v>0</v>
-      </c>
-      <c r="Z54">
-        <v>0</v>
-      </c>
-      <c r="AA54">
+      <c r="Y54" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z54" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA54" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6931,13 +6969,13 @@
       <c r="X55" t="s">
         <v>292</v>
       </c>
-      <c r="Y55">
-        <v>0</v>
-      </c>
-      <c r="Z55">
-        <v>0</v>
-      </c>
-      <c r="AA55">
+      <c r="Y55" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z55" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA55" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7014,13 +7052,13 @@
       <c r="X56" t="s">
         <v>296</v>
       </c>
-      <c r="Y56">
-        <v>1</v>
-      </c>
-      <c r="Z56">
-        <v>1</v>
-      </c>
-      <c r="AA56">
+      <c r="Y56" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z56" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA56" s="3">
         <v>1</v>
       </c>
     </row>
@@ -7097,13 +7135,13 @@
       <c r="X57" t="s">
         <v>300</v>
       </c>
-      <c r="Y57">
-        <v>0</v>
-      </c>
-      <c r="Z57">
-        <v>0</v>
-      </c>
-      <c r="AA57">
+      <c r="Y57" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z57" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA57" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7180,13 +7218,13 @@
       <c r="X58" t="s">
         <v>304</v>
       </c>
-      <c r="Y58">
-        <v>0</v>
-      </c>
-      <c r="Z58">
-        <v>0</v>
-      </c>
-      <c r="AA58">
+      <c r="Y58" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z58" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA58" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7263,13 +7301,13 @@
       <c r="X59" t="s">
         <v>308</v>
       </c>
-      <c r="Y59">
-        <v>1</v>
-      </c>
-      <c r="Z59">
-        <v>1</v>
-      </c>
-      <c r="AA59">
+      <c r="Y59" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z59" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA59" s="3">
         <v>1</v>
       </c>
     </row>
@@ -7346,13 +7384,13 @@
       <c r="X60" t="s">
         <v>312</v>
       </c>
-      <c r="Y60">
-        <v>0</v>
-      </c>
-      <c r="Z60">
-        <v>0</v>
-      </c>
-      <c r="AA60">
+      <c r="Y60" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z60" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA60" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7429,13 +7467,13 @@
       <c r="X61" t="s">
         <v>316</v>
       </c>
-      <c r="Y61">
-        <v>0</v>
-      </c>
-      <c r="Z61">
-        <v>0</v>
-      </c>
-      <c r="AA61">
+      <c r="Y61" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z61" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA61" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7512,13 +7550,13 @@
       <c r="X62" t="s">
         <v>320</v>
       </c>
-      <c r="Y62">
-        <v>1</v>
-      </c>
-      <c r="Z62">
-        <v>1</v>
-      </c>
-      <c r="AA62">
+      <c r="Y62" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z62" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA62" s="3">
         <v>1</v>
       </c>
     </row>
@@ -7595,13 +7633,13 @@
       <c r="X63" t="s">
         <v>324</v>
       </c>
-      <c r="Y63">
-        <v>0</v>
-      </c>
-      <c r="Z63">
-        <v>0</v>
-      </c>
-      <c r="AA63">
+      <c r="Y63" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z63" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA63" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7678,13 +7716,13 @@
       <c r="X64" t="s">
         <v>328</v>
       </c>
-      <c r="Y64">
-        <v>0</v>
-      </c>
-      <c r="Z64">
-        <v>0</v>
-      </c>
-      <c r="AA64">
+      <c r="Y64" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z64" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA64" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7761,13 +7799,13 @@
       <c r="X65" t="s">
         <v>332</v>
       </c>
-      <c r="Y65">
-        <v>1</v>
-      </c>
-      <c r="Z65">
-        <v>1</v>
-      </c>
-      <c r="AA65">
+      <c r="Y65" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z65" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA65" s="3">
         <v>1</v>
       </c>
     </row>
@@ -7844,13 +7882,13 @@
       <c r="X66" t="s">
         <v>336</v>
       </c>
-      <c r="Y66">
-        <v>0</v>
-      </c>
-      <c r="Z66">
-        <v>0</v>
-      </c>
-      <c r="AA66">
+      <c r="Y66" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z66" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA66" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7927,13 +7965,13 @@
       <c r="X67" t="s">
         <v>340</v>
       </c>
-      <c r="Y67">
-        <v>0</v>
-      </c>
-      <c r="Z67">
-        <v>0</v>
-      </c>
-      <c r="AA67">
+      <c r="Y67" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z67" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA67" s="3">
         <v>0</v>
       </c>
     </row>
@@ -8010,13 +8048,13 @@
       <c r="X68" t="s">
         <v>344</v>
       </c>
-      <c r="Y68">
-        <v>1</v>
-      </c>
-      <c r="Z68">
-        <v>1</v>
-      </c>
-      <c r="AA68">
+      <c r="Y68" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z68" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA68" s="3">
         <v>1</v>
       </c>
     </row>
@@ -8093,13 +8131,13 @@
       <c r="X69" t="s">
         <v>348</v>
       </c>
-      <c r="Y69">
-        <v>0</v>
-      </c>
-      <c r="Z69">
-        <v>0</v>
-      </c>
-      <c r="AA69">
+      <c r="Y69" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z69" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA69" s="3">
         <v>0</v>
       </c>
     </row>
@@ -8176,13 +8214,13 @@
       <c r="X70" t="s">
         <v>352</v>
       </c>
-      <c r="Y70">
-        <v>0</v>
-      </c>
-      <c r="Z70">
-        <v>0</v>
-      </c>
-      <c r="AA70">
+      <c r="Y70" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z70" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA70" s="3">
         <v>0</v>
       </c>
     </row>
@@ -8259,13 +8297,13 @@
       <c r="X71" t="s">
         <v>356</v>
       </c>
-      <c r="Y71">
-        <v>1</v>
-      </c>
-      <c r="Z71">
-        <v>1</v>
-      </c>
-      <c r="AA71">
+      <c r="Y71" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z71" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA71" s="3">
         <v>1</v>
       </c>
     </row>
@@ -8342,13 +8380,13 @@
       <c r="X72" t="s">
         <v>360</v>
       </c>
-      <c r="Y72">
-        <v>0</v>
-      </c>
-      <c r="Z72">
-        <v>0</v>
-      </c>
-      <c r="AA72">
+      <c r="Y72" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z72" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA72" s="3">
         <v>0</v>
       </c>
     </row>
@@ -8425,13 +8463,13 @@
       <c r="X73" t="s">
         <v>364</v>
       </c>
-      <c r="Y73">
-        <v>0</v>
-      </c>
-      <c r="Z73">
-        <v>0</v>
-      </c>
-      <c r="AA73">
+      <c r="Y73" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z73" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA73" s="3">
         <v>0</v>
       </c>
     </row>
@@ -8508,13 +8546,13 @@
       <c r="X74" t="s">
         <v>368</v>
       </c>
-      <c r="Y74">
-        <v>1</v>
-      </c>
-      <c r="Z74">
-        <v>1</v>
-      </c>
-      <c r="AA74">
+      <c r="Y74" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z74" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA74" s="3">
         <v>1</v>
       </c>
     </row>
@@ -8591,13 +8629,13 @@
       <c r="X75" t="s">
         <v>372</v>
       </c>
-      <c r="Y75">
-        <v>0</v>
-      </c>
-      <c r="Z75">
-        <v>0</v>
-      </c>
-      <c r="AA75">
+      <c r="Y75" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z75" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA75" s="3">
         <v>0</v>
       </c>
     </row>
@@ -8674,13 +8712,13 @@
       <c r="X76" t="s">
         <v>376</v>
       </c>
-      <c r="Y76">
-        <v>0</v>
-      </c>
-      <c r="Z76">
-        <v>0</v>
-      </c>
-      <c r="AA76">
+      <c r="Y76" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z76" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA76" s="3">
         <v>0</v>
       </c>
     </row>
@@ -8757,13 +8795,13 @@
       <c r="X77" t="s">
         <v>380</v>
       </c>
-      <c r="Y77">
-        <v>1</v>
-      </c>
-      <c r="Z77">
-        <v>1</v>
-      </c>
-      <c r="AA77">
+      <c r="Y77" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z77" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA77" s="3">
         <v>1</v>
       </c>
     </row>
@@ -8840,13 +8878,13 @@
       <c r="X78" t="s">
         <v>384</v>
       </c>
-      <c r="Y78">
-        <v>0</v>
-      </c>
-      <c r="Z78">
-        <v>0</v>
-      </c>
-      <c r="AA78">
+      <c r="Y78" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z78" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA78" s="3">
         <v>0</v>
       </c>
     </row>
@@ -8923,13 +8961,13 @@
       <c r="X79" t="s">
         <v>388</v>
       </c>
-      <c r="Y79">
-        <v>0</v>
-      </c>
-      <c r="Z79">
-        <v>0</v>
-      </c>
-      <c r="AA79">
+      <c r="Y79" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z79" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA79" s="3">
         <v>0</v>
       </c>
     </row>
@@ -9006,13 +9044,13 @@
       <c r="X80" t="s">
         <v>392</v>
       </c>
-      <c r="Y80">
-        <v>1</v>
-      </c>
-      <c r="Z80">
-        <v>1</v>
-      </c>
-      <c r="AA80">
+      <c r="Y80" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z80" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA80" s="3">
         <v>1</v>
       </c>
     </row>
@@ -9089,13 +9127,13 @@
       <c r="X81" t="s">
         <v>396</v>
       </c>
-      <c r="Y81">
-        <v>0</v>
-      </c>
-      <c r="Z81">
-        <v>0</v>
-      </c>
-      <c r="AA81">
+      <c r="Y81" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z81" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA81" s="3">
         <v>0</v>
       </c>
     </row>
@@ -9172,13 +9210,13 @@
       <c r="X82" t="s">
         <v>400</v>
       </c>
-      <c r="Y82">
-        <v>0</v>
-      </c>
-      <c r="Z82">
-        <v>0</v>
-      </c>
-      <c r="AA82">
+      <c r="Y82" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z82" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA82" s="3">
         <v>0</v>
       </c>
     </row>
@@ -9255,13 +9293,13 @@
       <c r="X83" t="s">
         <v>404</v>
       </c>
-      <c r="Y83">
-        <v>1</v>
-      </c>
-      <c r="Z83">
-        <v>1</v>
-      </c>
-      <c r="AA83">
+      <c r="Y83" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z83" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA83" s="3">
         <v>1</v>
       </c>
     </row>
@@ -9338,13 +9376,13 @@
       <c r="X84" t="s">
         <v>408</v>
       </c>
-      <c r="Y84">
-        <v>0</v>
-      </c>
-      <c r="Z84">
-        <v>0</v>
-      </c>
-      <c r="AA84">
+      <c r="Y84" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z84" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA84" s="3">
         <v>0</v>
       </c>
     </row>
@@ -9421,13 +9459,13 @@
       <c r="X85" t="s">
         <v>412</v>
       </c>
-      <c r="Y85">
-        <v>0</v>
-      </c>
-      <c r="Z85">
-        <v>0</v>
-      </c>
-      <c r="AA85">
+      <c r="Y85" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z85" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA85" s="3">
         <v>0</v>
       </c>
     </row>
@@ -9504,13 +9542,13 @@
       <c r="X86" t="s">
         <v>416</v>
       </c>
-      <c r="Y86">
-        <v>1</v>
-      </c>
-      <c r="Z86">
-        <v>1</v>
-      </c>
-      <c r="AA86">
+      <c r="Y86" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z86" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA86" s="3">
         <v>1</v>
       </c>
     </row>
@@ -9587,13 +9625,13 @@
       <c r="X87" t="s">
         <v>420</v>
       </c>
-      <c r="Y87">
-        <v>0</v>
-      </c>
-      <c r="Z87">
-        <v>0</v>
-      </c>
-      <c r="AA87">
+      <c r="Y87" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z87" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA87" s="3">
         <v>0</v>
       </c>
     </row>
@@ -9670,13 +9708,13 @@
       <c r="X88" t="s">
         <v>424</v>
       </c>
-      <c r="Y88">
-        <v>0</v>
-      </c>
-      <c r="Z88">
-        <v>0</v>
-      </c>
-      <c r="AA88">
+      <c r="Y88" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z88" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA88" s="3">
         <v>0</v>
       </c>
     </row>
@@ -9753,13 +9791,13 @@
       <c r="X89" t="s">
         <v>428</v>
       </c>
-      <c r="Y89">
-        <v>1</v>
-      </c>
-      <c r="Z89">
-        <v>1</v>
-      </c>
-      <c r="AA89">
+      <c r="Y89" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z89" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA89" s="3">
         <v>1</v>
       </c>
     </row>
@@ -9836,13 +9874,13 @@
       <c r="X90" t="s">
         <v>432</v>
       </c>
-      <c r="Y90">
-        <v>0</v>
-      </c>
-      <c r="Z90">
-        <v>0</v>
-      </c>
-      <c r="AA90">
+      <c r="Y90" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z90" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA90" s="3">
         <v>0</v>
       </c>
     </row>
@@ -9919,13 +9957,13 @@
       <c r="X91" t="s">
         <v>436</v>
       </c>
-      <c r="Y91">
-        <v>0</v>
-      </c>
-      <c r="Z91">
-        <v>0</v>
-      </c>
-      <c r="AA91">
+      <c r="Y91" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z91" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA91" s="3">
         <v>0</v>
       </c>
     </row>
@@ -10002,13 +10040,13 @@
       <c r="X92" t="s">
         <v>440</v>
       </c>
-      <c r="Y92">
-        <v>1</v>
-      </c>
-      <c r="Z92">
-        <v>1</v>
-      </c>
-      <c r="AA92">
+      <c r="Y92" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z92" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA92" s="3">
         <v>1</v>
       </c>
     </row>
@@ -10085,13 +10123,13 @@
       <c r="X93" t="s">
         <v>444</v>
       </c>
-      <c r="Y93">
-        <v>0</v>
-      </c>
-      <c r="Z93">
-        <v>0</v>
-      </c>
-      <c r="AA93">
+      <c r="Y93" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z93" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA93" s="3">
         <v>0</v>
       </c>
     </row>
@@ -10168,13 +10206,13 @@
       <c r="X94" t="s">
         <v>448</v>
       </c>
-      <c r="Y94">
-        <v>0</v>
-      </c>
-      <c r="Z94">
-        <v>0</v>
-      </c>
-      <c r="AA94">
+      <c r="Y94" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z94" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA94" s="3">
         <v>0</v>
       </c>
     </row>
@@ -10251,13 +10289,13 @@
       <c r="X95" t="s">
         <v>452</v>
       </c>
-      <c r="Y95">
-        <v>1</v>
-      </c>
-      <c r="Z95">
-        <v>1</v>
-      </c>
-      <c r="AA95">
+      <c r="Y95" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z95" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA95" s="3">
         <v>1</v>
       </c>
     </row>
@@ -10334,13 +10372,13 @@
       <c r="X96" t="s">
         <v>456</v>
       </c>
-      <c r="Y96">
-        <v>0</v>
-      </c>
-      <c r="Z96">
-        <v>0</v>
-      </c>
-      <c r="AA96">
+      <c r="Y96" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z96" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA96" s="3">
         <v>0</v>
       </c>
     </row>
@@ -10417,13 +10455,13 @@
       <c r="X97" t="s">
         <v>460</v>
       </c>
-      <c r="Y97">
-        <v>0</v>
-      </c>
-      <c r="Z97">
-        <v>0</v>
-      </c>
-      <c r="AA97">
+      <c r="Y97" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z97" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA97" s="3">
         <v>0</v>
       </c>
     </row>
@@ -10500,13 +10538,13 @@
       <c r="X98" t="s">
         <v>464</v>
       </c>
-      <c r="Y98">
-        <v>1</v>
-      </c>
-      <c r="Z98">
-        <v>1</v>
-      </c>
-      <c r="AA98">
+      <c r="Y98" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z98" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA98" s="3">
         <v>1</v>
       </c>
     </row>
@@ -10583,13 +10621,13 @@
       <c r="X99" t="s">
         <v>468</v>
       </c>
-      <c r="Y99">
-        <v>0</v>
-      </c>
-      <c r="Z99">
-        <v>0</v>
-      </c>
-      <c r="AA99">
+      <c r="Y99" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z99" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA99" s="3">
         <v>0</v>
       </c>
     </row>
@@ -10666,13 +10704,13 @@
       <c r="X100" t="s">
         <v>472</v>
       </c>
-      <c r="Y100">
-        <v>0</v>
-      </c>
-      <c r="Z100">
-        <v>0</v>
-      </c>
-      <c r="AA100">
+      <c r="Y100" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z100" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA100" s="3">
         <v>0</v>
       </c>
     </row>
@@ -10749,13 +10787,13 @@
       <c r="X101" t="s">
         <v>476</v>
       </c>
-      <c r="Y101">
-        <v>1</v>
-      </c>
-      <c r="Z101">
-        <v>1</v>
-      </c>
-      <c r="AA101">
+      <c r="Y101" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z101" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA101" s="3">
         <v>1</v>
       </c>
     </row>
@@ -10832,13 +10870,13 @@
       <c r="X102" t="s">
         <v>480</v>
       </c>
-      <c r="Y102">
-        <v>0</v>
-      </c>
-      <c r="Z102">
-        <v>0</v>
-      </c>
-      <c r="AA102">
+      <c r="Y102" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z102" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA102" s="3">
         <v>0</v>
       </c>
     </row>
@@ -10915,13 +10953,13 @@
       <c r="X103" t="s">
         <v>484</v>
       </c>
-      <c r="Y103">
-        <v>0</v>
-      </c>
-      <c r="Z103">
-        <v>0</v>
-      </c>
-      <c r="AA103">
+      <c r="Y103" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z103" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA103" s="3">
         <v>0</v>
       </c>
     </row>
@@ -10998,13 +11036,13 @@
       <c r="X104" t="s">
         <v>488</v>
       </c>
-      <c r="Y104">
-        <v>1</v>
-      </c>
-      <c r="Z104">
-        <v>1</v>
-      </c>
-      <c r="AA104">
+      <c r="Y104" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z104" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA104" s="3">
         <v>1</v>
       </c>
     </row>
@@ -11081,13 +11119,13 @@
       <c r="X105" t="s">
         <v>492</v>
       </c>
-      <c r="Y105">
-        <v>0</v>
-      </c>
-      <c r="Z105">
-        <v>0</v>
-      </c>
-      <c r="AA105">
+      <c r="Y105" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z105" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA105" s="3">
         <v>0</v>
       </c>
     </row>
@@ -11164,13 +11202,13 @@
       <c r="X106" t="s">
         <v>496</v>
       </c>
-      <c r="Y106">
-        <v>0</v>
-      </c>
-      <c r="Z106">
-        <v>0</v>
-      </c>
-      <c r="AA106">
+      <c r="Y106" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z106" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA106" s="3">
         <v>0</v>
       </c>
     </row>
@@ -11247,13 +11285,13 @@
       <c r="X107" t="s">
         <v>500</v>
       </c>
-      <c r="Y107">
-        <v>1</v>
-      </c>
-      <c r="Z107">
-        <v>1</v>
-      </c>
-      <c r="AA107">
+      <c r="Y107" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z107" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA107" s="3">
         <v>1</v>
       </c>
     </row>
@@ -11330,13 +11368,13 @@
       <c r="X108" t="s">
         <v>504</v>
       </c>
-      <c r="Y108">
-        <v>0</v>
-      </c>
-      <c r="Z108">
-        <v>0</v>
-      </c>
-      <c r="AA108">
+      <c r="Y108" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z108" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA108" s="3">
         <v>0</v>
       </c>
     </row>
@@ -11413,13 +11451,13 @@
       <c r="X109" t="s">
         <v>508</v>
       </c>
-      <c r="Y109">
-        <v>0</v>
-      </c>
-      <c r="Z109">
-        <v>0</v>
-      </c>
-      <c r="AA109">
+      <c r="Y109" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z109" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA109" s="3">
         <v>0</v>
       </c>
     </row>
@@ -11496,13 +11534,13 @@
       <c r="X110" t="s">
         <v>512</v>
       </c>
-      <c r="Y110">
-        <v>1</v>
-      </c>
-      <c r="Z110">
-        <v>1</v>
-      </c>
-      <c r="AA110">
+      <c r="Y110" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z110" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA110" s="3">
         <v>1</v>
       </c>
     </row>
@@ -11579,13 +11617,13 @@
       <c r="X111" t="s">
         <v>516</v>
       </c>
-      <c r="Y111">
-        <v>0</v>
-      </c>
-      <c r="Z111">
-        <v>0</v>
-      </c>
-      <c r="AA111">
+      <c r="Y111" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z111" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA111" s="3">
         <v>0</v>
       </c>
     </row>
@@ -11662,13 +11700,13 @@
       <c r="X112" t="s">
         <v>519</v>
       </c>
-      <c r="Y112">
-        <v>0</v>
-      </c>
-      <c r="Z112">
-        <v>0</v>
-      </c>
-      <c r="AA112">
+      <c r="Y112" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z112" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA112" s="3">
         <v>0</v>
       </c>
     </row>
@@ -11745,13 +11783,13 @@
       <c r="X113" t="s">
         <v>523</v>
       </c>
-      <c r="Y113">
-        <v>1</v>
-      </c>
-      <c r="Z113">
-        <v>1</v>
-      </c>
-      <c r="AA113">
+      <c r="Y113" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z113" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA113" s="3">
         <v>1</v>
       </c>
     </row>
@@ -11828,13 +11866,13 @@
       <c r="X114" t="s">
         <v>527</v>
       </c>
-      <c r="Y114">
-        <v>0</v>
-      </c>
-      <c r="Z114">
-        <v>0</v>
-      </c>
-      <c r="AA114">
+      <c r="Y114" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z114" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA114" s="3">
         <v>0</v>
       </c>
     </row>
@@ -11911,13 +11949,13 @@
       <c r="X115" t="s">
         <v>531</v>
       </c>
-      <c r="Y115">
-        <v>0</v>
-      </c>
-      <c r="Z115">
-        <v>0</v>
-      </c>
-      <c r="AA115">
+      <c r="Y115" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z115" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA115" s="3">
         <v>0</v>
       </c>
     </row>
@@ -11994,13 +12032,13 @@
       <c r="X116" t="s">
         <v>535</v>
       </c>
-      <c r="Y116">
-        <v>1</v>
-      </c>
-      <c r="Z116">
-        <v>1</v>
-      </c>
-      <c r="AA116">
+      <c r="Y116" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z116" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA116" s="3">
         <v>1</v>
       </c>
     </row>
@@ -12077,13 +12115,13 @@
       <c r="X117" t="s">
         <v>539</v>
       </c>
-      <c r="Y117">
-        <v>0</v>
-      </c>
-      <c r="Z117">
-        <v>0</v>
-      </c>
-      <c r="AA117">
+      <c r="Y117" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z117" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA117" s="3">
         <v>0</v>
       </c>
     </row>
@@ -12160,13 +12198,13 @@
       <c r="X118" t="s">
         <v>543</v>
       </c>
-      <c r="Y118">
-        <v>0</v>
-      </c>
-      <c r="Z118">
-        <v>0</v>
-      </c>
-      <c r="AA118">
+      <c r="Y118" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z118" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA118" s="3">
         <v>0</v>
       </c>
     </row>
@@ -12243,13 +12281,13 @@
       <c r="X119" t="s">
         <v>547</v>
       </c>
-      <c r="Y119">
-        <v>1</v>
-      </c>
-      <c r="Z119">
-        <v>1</v>
-      </c>
-      <c r="AA119">
+      <c r="Y119" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z119" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA119" s="3">
         <v>1</v>
       </c>
     </row>
@@ -12326,13 +12364,13 @@
       <c r="X120" t="s">
         <v>551</v>
       </c>
-      <c r="Y120">
-        <v>0</v>
-      </c>
-      <c r="Z120">
-        <v>0</v>
-      </c>
-      <c r="AA120">
+      <c r="Y120" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z120" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA120" s="3">
         <v>0</v>
       </c>
     </row>
@@ -12409,13 +12447,13 @@
       <c r="X121" t="s">
         <v>555</v>
       </c>
-      <c r="Y121">
-        <v>0</v>
-      </c>
-      <c r="Z121">
-        <v>0</v>
-      </c>
-      <c r="AA121">
+      <c r="Y121" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z121" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA121" s="3">
         <v>0</v>
       </c>
     </row>
@@ -12492,13 +12530,13 @@
       <c r="X122" t="s">
         <v>559</v>
       </c>
-      <c r="Y122">
-        <v>1</v>
-      </c>
-      <c r="Z122">
-        <v>1</v>
-      </c>
-      <c r="AA122">
+      <c r="Y122" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z122" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA122" s="3">
         <v>1</v>
       </c>
     </row>
@@ -12575,13 +12613,13 @@
       <c r="X123" t="s">
         <v>563</v>
       </c>
-      <c r="Y123">
-        <v>0</v>
-      </c>
-      <c r="Z123">
-        <v>0</v>
-      </c>
-      <c r="AA123">
+      <c r="Y123" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z123" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA123" s="3">
         <v>0</v>
       </c>
     </row>
@@ -12658,13 +12696,13 @@
       <c r="X124" t="s">
         <v>567</v>
       </c>
-      <c r="Y124">
-        <v>0</v>
-      </c>
-      <c r="Z124">
-        <v>0</v>
-      </c>
-      <c r="AA124">
+      <c r="Y124" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z124" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA124" s="3">
         <v>0</v>
       </c>
     </row>
@@ -12741,13 +12779,13 @@
       <c r="X125" t="s">
         <v>571</v>
       </c>
-      <c r="Y125">
-        <v>1</v>
-      </c>
-      <c r="Z125">
-        <v>1</v>
-      </c>
-      <c r="AA125">
+      <c r="Y125" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z125" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA125" s="3">
         <v>1</v>
       </c>
     </row>
@@ -12824,13 +12862,13 @@
       <c r="X126" t="s">
         <v>575</v>
       </c>
-      <c r="Y126">
-        <v>0</v>
-      </c>
-      <c r="Z126">
-        <v>0</v>
-      </c>
-      <c r="AA126">
+      <c r="Y126" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z126" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA126" s="3">
         <v>0</v>
       </c>
     </row>
@@ -12907,13 +12945,13 @@
       <c r="X127" t="s">
         <v>579</v>
       </c>
-      <c r="Y127">
-        <v>0</v>
-      </c>
-      <c r="Z127">
-        <v>0</v>
-      </c>
-      <c r="AA127">
+      <c r="Y127" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z127" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA127" s="3">
         <v>0</v>
       </c>
     </row>
@@ -12990,13 +13028,13 @@
       <c r="X128" t="s">
         <v>583</v>
       </c>
-      <c r="Y128">
-        <v>1</v>
-      </c>
-      <c r="Z128">
-        <v>1</v>
-      </c>
-      <c r="AA128">
+      <c r="Y128" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z128" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA128" s="3">
         <v>1</v>
       </c>
     </row>
@@ -13073,13 +13111,13 @@
       <c r="X129" t="s">
         <v>587</v>
       </c>
-      <c r="Y129">
-        <v>0</v>
-      </c>
-      <c r="Z129">
-        <v>0</v>
-      </c>
-      <c r="AA129">
+      <c r="Y129" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z129" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA129" s="3">
         <v>0</v>
       </c>
     </row>
@@ -13156,13 +13194,13 @@
       <c r="X130" t="s">
         <v>591</v>
       </c>
-      <c r="Y130">
-        <v>0</v>
-      </c>
-      <c r="Z130">
-        <v>0</v>
-      </c>
-      <c r="AA130">
+      <c r="Y130" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z130" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA130" s="3">
         <v>0</v>
       </c>
     </row>
@@ -13239,13 +13277,13 @@
       <c r="X131" t="s">
         <v>595</v>
       </c>
-      <c r="Y131">
-        <v>1</v>
-      </c>
-      <c r="Z131">
-        <v>1</v>
-      </c>
-      <c r="AA131">
+      <c r="Y131" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z131" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA131" s="3">
         <v>1</v>
       </c>
     </row>
@@ -13322,13 +13360,13 @@
       <c r="X132" t="s">
         <v>599</v>
       </c>
-      <c r="Y132">
-        <v>0</v>
-      </c>
-      <c r="Z132">
-        <v>0</v>
-      </c>
-      <c r="AA132">
+      <c r="Y132" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z132" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA132" s="3">
         <v>0</v>
       </c>
     </row>
@@ -13405,13 +13443,13 @@
       <c r="X133" t="s">
         <v>603</v>
       </c>
-      <c r="Y133">
-        <v>0</v>
-      </c>
-      <c r="Z133">
-        <v>0</v>
-      </c>
-      <c r="AA133">
+      <c r="Y133" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z133" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA133" s="3">
         <v>0</v>
       </c>
     </row>
@@ -13488,13 +13526,13 @@
       <c r="X134" t="s">
         <v>607</v>
       </c>
-      <c r="Y134">
-        <v>1</v>
-      </c>
-      <c r="Z134">
-        <v>1</v>
-      </c>
-      <c r="AA134">
+      <c r="Y134" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z134" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA134" s="3">
         <v>1</v>
       </c>
     </row>
@@ -13571,13 +13609,13 @@
       <c r="X135" t="s">
         <v>611</v>
       </c>
-      <c r="Y135">
-        <v>0</v>
-      </c>
-      <c r="Z135">
-        <v>0</v>
-      </c>
-      <c r="AA135">
+      <c r="Y135" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z135" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA135" s="3">
         <v>0</v>
       </c>
     </row>
@@ -13654,13 +13692,13 @@
       <c r="X136" t="s">
         <v>615</v>
       </c>
-      <c r="Y136">
-        <v>0</v>
-      </c>
-      <c r="Z136">
-        <v>0</v>
-      </c>
-      <c r="AA136">
+      <c r="Y136" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z136" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA136" s="3">
         <v>0</v>
       </c>
     </row>
@@ -13737,13 +13775,13 @@
       <c r="X137" t="s">
         <v>619</v>
       </c>
-      <c r="Y137">
-        <v>1</v>
-      </c>
-      <c r="Z137">
-        <v>1</v>
-      </c>
-      <c r="AA137">
+      <c r="Y137" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z137" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA137" s="3">
         <v>1</v>
       </c>
     </row>
@@ -13820,13 +13858,13 @@
       <c r="X138" t="s">
         <v>623</v>
       </c>
-      <c r="Y138">
-        <v>0</v>
-      </c>
-      <c r="Z138">
-        <v>0</v>
-      </c>
-      <c r="AA138">
+      <c r="Y138" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z138" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA138" s="3">
         <v>0</v>
       </c>
     </row>
@@ -13903,13 +13941,13 @@
       <c r="X139" t="s">
         <v>627</v>
       </c>
-      <c r="Y139">
-        <v>0</v>
-      </c>
-      <c r="Z139">
-        <v>0</v>
-      </c>
-      <c r="AA139">
+      <c r="Y139" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z139" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA139" s="3">
         <v>0</v>
       </c>
     </row>
@@ -13986,13 +14024,13 @@
       <c r="X140" t="s">
         <v>631</v>
       </c>
-      <c r="Y140">
-        <v>1</v>
-      </c>
-      <c r="Z140">
-        <v>1</v>
-      </c>
-      <c r="AA140">
+      <c r="Y140" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z140" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA140" s="3">
         <v>1</v>
       </c>
     </row>
@@ -14069,13 +14107,13 @@
       <c r="X141" t="s">
         <v>635</v>
       </c>
-      <c r="Y141">
-        <v>0</v>
-      </c>
-      <c r="Z141">
-        <v>0</v>
-      </c>
-      <c r="AA141">
+      <c r="Y141" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z141" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA141" s="3">
         <v>0</v>
       </c>
     </row>
@@ -14152,13 +14190,13 @@
       <c r="X142" t="s">
         <v>639</v>
       </c>
-      <c r="Y142">
-        <v>0</v>
-      </c>
-      <c r="Z142">
-        <v>0</v>
-      </c>
-      <c r="AA142">
+      <c r="Y142" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z142" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA142" s="3">
         <v>0</v>
       </c>
     </row>
@@ -14235,13 +14273,13 @@
       <c r="X143" t="s">
         <v>643</v>
       </c>
-      <c r="Y143">
-        <v>1</v>
-      </c>
-      <c r="Z143">
-        <v>1</v>
-      </c>
-      <c r="AA143">
+      <c r="Y143" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z143" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA143" s="3">
         <v>1</v>
       </c>
     </row>
@@ -14318,13 +14356,13 @@
       <c r="X144" t="s">
         <v>647</v>
       </c>
-      <c r="Y144">
-        <v>0</v>
-      </c>
-      <c r="Z144">
-        <v>0</v>
-      </c>
-      <c r="AA144">
+      <c r="Y144" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z144" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA144" s="3">
         <v>0</v>
       </c>
     </row>
@@ -14401,13 +14439,13 @@
       <c r="X145" t="s">
         <v>651</v>
       </c>
-      <c r="Y145">
-        <v>0</v>
-      </c>
-      <c r="Z145">
-        <v>0</v>
-      </c>
-      <c r="AA145">
+      <c r="Y145" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z145" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA145" s="3">
         <v>0</v>
       </c>
     </row>
@@ -14484,13 +14522,13 @@
       <c r="X146" t="s">
         <v>655</v>
       </c>
-      <c r="Y146">
-        <v>1</v>
-      </c>
-      <c r="Z146">
-        <v>1</v>
-      </c>
-      <c r="AA146">
+      <c r="Y146" s="3">
+        <v>1</v>
+      </c>
+      <c r="Z146" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA146" s="3">
         <v>1</v>
       </c>
     </row>
@@ -14567,13 +14605,13 @@
       <c r="X147" t="s">
         <v>659</v>
       </c>
-      <c r="Y147">
-        <v>0</v>
-      </c>
-      <c r="Z147">
-        <v>0</v>
-      </c>
-      <c r="AA147">
+      <c r="Y147" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z147" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA147" s="3">
         <v>0</v>
       </c>
     </row>
@@ -14650,13 +14688,13 @@
       <c r="X148" t="s">
         <v>663</v>
       </c>
-      <c r="Y148">
-        <v>0</v>
-      </c>
-      <c r="Z148">
-        <v>0</v>
-      </c>
-      <c r="AA148">
+      <c r="Y148" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z148" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA148" s="3">
         <v>0</v>
       </c>
     </row>

</xml_diff>